<commit_message>
fix(017A): close cancel bypass, style Excel template, durable preview UX
Round4: block model excelWorkflowCancel; human summaries; Redis preview follow-up for 入库吧; local 10/10+14/14 no-post.
</commit_message>
<xml_diff>
--- a/docs/poc/evidence/采购入库模板---100L---.xlsx
+++ b/docs/poc/evidence/采购入库模板---100L---.xlsx
@@ -9,22 +9,40 @@
     <sheet name="使用说明" r:id="rId3" sheetId="1"/>
     <sheet name="02采购入库" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'02采购入库'!$A$3:$J$4</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>AI-ERP 演示 Excel。第3行是表头，第4行起是数据。配比为虚构测试数据，不是化学工艺。</t>
-  </si>
-  <si>
-    <t>上传只生成预览。库存变化只发生在用户确认之后。物料期初和销售出库仅供下载，不能经本网关确认。</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+  <si>
+    <t>AI-ERP 企微业务模板（与 jshERP 原生 .xls 导入格式不同，请用本模板）</t>
+  </si>
+  <si>
+    <t>第3行是表头（勿改列名），第4行起填数据。红色表头=必填，灰色表头=选填。</t>
+  </si>
+  <si>
+    <t>同一「业务单号/配制单号/服务单号」多行 = 同一张单的多条明细；换单号即新单。</t>
+  </si>
+  <si>
+    <t>已预填唯一单号与当天日期，请补齐供应商/物料/数量等；勿编造无权仓库或供应商。</t>
+  </si>
+  <si>
+    <t>不要使用公式或宏。上传后只做核对预览，确认入库前库存不变。</t>
+  </si>
+  <si>
+    <t>示例（请勿当作真实业务粘贴）：采购单号 CG-20261021-DEMO｜原料仓｜RM-A001｜10 L。</t>
+  </si>
+  <si>
+    <t>销售出库/物料期初当前仅提供模板，不能经本流程确认过账。</t>
   </si>
   <si>
     <t>02采购入库</t>
   </si>
   <si>
-    <t>第3行表头，第4行开始填写。不要使用公式。</t>
+    <t>红色必填：业务单号、业务日期、供应商、物料编码、入库仓库、入库数量、单位。同单号多行=同一张采购单。勿用公式。</t>
   </si>
   <si>
     <t>业务单号</t>
@@ -92,7 +110,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -100,16 +118,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="14.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <color indexed="23"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="43"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,20 +167,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="70.3125" customWidth="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -142,6 +206,31 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -151,82 +240,103 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="16.40625" customWidth="true"/>
+    <col min="2" max="2" width="13.28125" customWidth="true"/>
+    <col min="3" max="3" width="17.578125" customWidth="true"/>
+    <col min="4" max="4" width="16.40625" customWidth="true"/>
+    <col min="5" max="5" width="17.578125" customWidth="true"/>
+    <col min="6" max="6" width="13.28125" customWidth="true"/>
+    <col min="7" max="7" width="13.28125" customWidth="true"/>
+    <col min="8" max="8" width="13.28125" customWidth="true"/>
+    <col min="9" max="9" width="13.28125" customWidth="true"/>
+    <col min="10" max="10" width="17.578125" customWidth="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>2</v>
+      <c r="A1" t="s" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>3</v>
+      <c r="A2" t="s" s="4">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="A3" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="G3" t="s">
+      <c r="B3" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="H3" t="s">
+      <c r="C3" t="s" s="2">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
+      <c r="D3" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="J3" t="s">
+      <c r="E3" t="s" s="3">
         <v>13</v>
+      </c>
+      <c r="F3" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s" s="3">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s" s="3">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:J4"/>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="F4:F201" allowBlank="true" errorStyle="stop" showDropDown="true" showErrorMessage="true">
+      <formula1>"原料仓,成品仓"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="H4:H201" allowBlank="true" errorStyle="stop" showDropDown="true" showErrorMessage="true">
+      <formula1>"L,kg,g,个,瓶,箱,桶"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>